<commit_message>
4742 - Adjust Cobra Precision
</commit_message>
<xml_diff>
--- a/GenBOE/RDM.Web/Templates/Export/CobraExport.xlsx
+++ b/GenBOE/RDM.Web/Templates/Export/CobraExport.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="21929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C326EE-6F2C-49B9-8A6D-60C4D8014C26}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,12 +35,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-    <numFmt numFmtId="165" formatCode="0.00000"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -53,13 +54,71 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF452DB2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070729"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9F9F9F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF452DB2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD35714"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -71,8 +130,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -80,8 +145,14 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="PPDuplicateRow" xfId="4" xr:uid="{E6A63F5F-7410-48E8-997A-361CC18EE29D}"/>
+    <cellStyle name="PPHeaderColumn" xfId="2" xr:uid="{0F1C63B9-A001-49B5-8CF2-4DB9DD8E2C4B}"/>
+    <cellStyle name="PPHeaderRequired" xfId="3" xr:uid="{75AEED5F-79F2-4645-A244-5167DC6D96BB}"/>
+    <cellStyle name="PPHeaderTop" xfId="1" xr:uid="{8F09E9FC-2A02-4961-8EB4-EF1E8896109B}"/>
+    <cellStyle name="PPInvalidValue" xfId="5" xr:uid="{FC13FC4F-878E-448D-BA18-FE016FD874C4}"/>
+    <cellStyle name="PPMissingValue" xfId="6" xr:uid="{B53D3A1C-194C-45A8-8D51-CB1A83A8832A}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -172,6 +243,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -207,6 +295,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -382,7 +487,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -390,7 +495,7 @@
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="31.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="3" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -414,5 +519,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C_x000D__x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D__x000D_</oddFooter>
+    <evenHeader>&amp;C_x000D__x000D_</evenHeader>
+    <evenFooter>&amp;C_x000D__x000D_</evenFooter>
+    <firstHeader>&amp;C_x000D__x000D_</firstHeader>
+    <firstFooter>&amp;C_x000D__x000D_</firstFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>